<commit_message>
Update 3D model transfer issues table with print-specific fixes
Added 3D print transfer issues section covering scale mismatch,
non-manifold geometry, unapplied modifiers, inverted faces, low-res
mesh, and file format errors with symptoms, fixes, and tools.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3D_Model_Transfer_Issues.xlsx
+++ b/3D_Model_Transfer_Issues.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,264 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>3D Print Transfer Issues &amp; Fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Symptom</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Tools / Notes</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Export Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Incorrect Scale / Size</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Scale Mismatch</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Model appears tiny or massive in the slicer.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Set modeling software to Metric (mm) before exporting. Set 1 Blender unit = 1 mm.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Blender Unit settings, slicer scale tool</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Verify units match between modeler and slicer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Non-Manifold Geometry</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Mesh Errors</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Missing faces, holes, or edges shared by more than two faces — model is unprintable.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Use repair software to fill holes and fix mesh errors.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>3D Builder, Meshmixer, Netfabb</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Run mesh analysis before export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Unapplied Modifiers</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Export Oversight</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Mirror, Solidify, or Boolean modifiers don't carry over to the exported STL.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Apply all modifiers in the modeling software before exporting.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Blender: Ctrl+A modifiers</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Check modifier stack is empty before export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Intersecting / Inverted Faces</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Normal Errors</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Faces are inside out or intersecting, causing slicer errors.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Recalculate normals (Flip / Align Normals) in the modeling program.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Blender: Shift+N recalculate outside</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Enable face orientation overlay to spot issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Low Resolution Mesh</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Mesh Quality</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Curved surfaces appear blocky or angular (faceted look).</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Increase subdivision or export resolution in exporter settings.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Subdivision Surface modifier</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Balance poly count vs. file size for your printer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>File Format Errors</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Compatibility</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>STL file not recognized, or ASCII vs. Binary STL mismatch.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Use Binary STL for smaller files and better compatibility. Ensure .stl extension.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Most slicers prefer Binary STL</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Binary STL is the safer default for all printers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:G6"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>